<commit_message>
Correct the MPN for a resistor/ Added NLNet and OSHW logos
</commit_message>
<xml_diff>
--- a/RASRF2400WBMC/Hardware/Production/RevA.0/BoM/RASRF2400WBMC_BoM.xlsx
+++ b/RASRF2400WBMC/Hardware/Production/RevA.0/BoM/RASRF2400WBMC_BoM.xlsx
@@ -469,7 +469,7 @@
     <t xml:space="preserve">U2</t>
   </si>
   <si>
-    <t xml:space="preserve">LD1117DT18</t>
+    <t xml:space="preserve">LD1117DT33TR</t>
   </si>
   <si>
     <t xml:space="preserve">DPAK456P1010X240-3N</t>
@@ -478,10 +478,7 @@
     <t xml:space="preserve">STMicroelectronics</t>
   </si>
   <si>
-    <t xml:space="preserve">LD1117DT18CTR, LD1117DT18TR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IC, LDO Regulator, 1.8V, 800mA, Fixed, DPAK (TO-252), T&amp;R</t>
+    <t xml:space="preserve">IC, LDO Regulator, 3.3V, 800mA, Fixed, DPAK (TO-252), T&amp;R</t>
   </si>
   <si>
     <t xml:space="preserve">U4,U6,U8,U10</t>
@@ -548,6 +545,9 @@
   </si>
   <si>
     <t xml:space="preserve">100K</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0402FR-07100KL</t>
   </si>
   <si>
     <t xml:space="preserve">Res, Thick Film, 100kΩ, 1/16W, 0402, ±1%</t>
@@ -813,12 +813,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1015,7 +1019,7 @@
   <dimension ref="A1:J62"/>
   <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="11" min="11" style="0" width="58.43"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.88"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1854,151 +1858,151 @@
         <v>151</v>
       </c>
       <c r="I37" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="J37" s="1" t="s">
         <v>152</v>
-      </c>
-      <c r="J37" s="1" t="s">
-        <v>153</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="1" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B38" s="1" t="n">
         <v>4</v>
       </c>
       <c r="C38" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="G38" s="1" t="s">
         <v>155</v>
       </c>
-      <c r="G38" s="1" t="s">
+      <c r="H38" s="1" t="s">
         <v>156</v>
       </c>
-      <c r="H38" s="1" t="s">
+      <c r="I38" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="J38" s="1" t="s">
         <v>157</v>
-      </c>
-      <c r="I38" s="1" t="s">
-        <v>155</v>
-      </c>
-      <c r="J38" s="1" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B39" s="1" t="n">
         <v>1</v>
       </c>
       <c r="C39" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="G39" s="1" t="s">
         <v>160</v>
       </c>
-      <c r="G39" s="1" t="s">
+      <c r="H39" s="1" t="s">
         <v>161</v>
       </c>
-      <c r="H39" s="1" t="s">
+      <c r="I39" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="J39" s="1" t="s">
         <v>162</v>
-      </c>
-      <c r="I39" s="1" t="s">
-        <v>160</v>
-      </c>
-      <c r="J39" s="1" t="s">
-        <v>163</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B40" s="1" t="n">
         <v>14</v>
       </c>
       <c r="C40" s="1" t="s">
+        <v>164</v>
+      </c>
+      <c r="G40" s="1" t="s">
         <v>165</v>
-      </c>
-      <c r="G40" s="1" t="s">
-        <v>166</v>
       </c>
       <c r="H40" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I40" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="J40" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="J40" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="1" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B41" s="1" t="n">
         <v>8</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D41" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H41" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I41" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="J41" s="1" t="s">
         <v>167</v>
-      </c>
-      <c r="J41" s="1" t="s">
-        <v>168</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="1" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B42" s="1" t="n">
         <v>2</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D42" s="1" t="s">
         <v>3</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I42" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="J42" s="1" t="s">
         <v>172</v>
       </c>
-      <c r="J42" s="1" t="s">
+    </row>
+    <row r="43" s="2" customFormat="true" ht="19.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
         <v>173</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="1" t="s">
-        <v>174</v>
       </c>
       <c r="B43" s="1" t="n">
         <v>5</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G43" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="H43" s="1" t="s">
         <v>87</v>
       </c>
       <c r="I43" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="J43" s="1" t="s">
         <v>176</v>
@@ -2035,7 +2039,7 @@
         <v>1</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D45" s="1" t="s">
         <v>3</v>
@@ -2061,7 +2065,7 @@
         <v>2</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="G46" s="1" t="s">
         <v>179</v>
@@ -2107,7 +2111,7 @@
         <v>1</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="G48" s="1" t="s">
         <v>179</v>
@@ -2130,7 +2134,7 @@
         <v>1</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D49" s="1" t="s">
         <v>3</v>

</xml_diff>